<commit_message>
khám phá dữ liệu
</commit_message>
<xml_diff>
--- a/house_price_ml/07_logs/change_log.xlsx
+++ b/house_price_ml/07_logs/change_log.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="375">
   <si>
     <t xml:space="preserve">change_log.xlsx - Nhật ký thay đổi dự án ML</t>
   </si>
@@ -423,6 +423,219 @@
     <t xml:space="preserve">Đính chính đánh số bước: dòng LOG-0016/LOG-0017 (chạy make_splits.py, copy script) được ghi với step-label 'P2 Chia train/val/test' do đánh số nhầm; đúng theo quy trình skill thì bước chia dữ liệu là P3, không phải P2. Không sửa lại các dòng cũ đó (append-only), chỉ đính chính tại đây.</t>
   </si>
   <si>
+    <t xml:space="preserve">LOG-0020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2.5 Khám phá dữ liệu (EDA, chỉ trên train)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chạy EDA chỉ trên split=='train' của 01_data/splits/split_v1.csv (1022 dòng), tuân thủ nguyên tắc 'EDA chỉ trên train' của skill. Xem: phân phối SalePrice, missing (đối chiếu số liệu với audit toàn bộ), tương quan numeric, quét ngoại lai IQR, mức hạng mục hiếm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SalePrice train: skew=1.73 (log1p skew=0.15, xác nhận log-transform hợp lý). Missing top: PoolQC 99.4%, MiscFeature 96.0%, Alley 93.4%, Fence 80.2%, MasVnrType 59.2%, FireplaceQu 47.1% - khớp tỉ lệ với audit toàn bộ (P1), xác nhận split không lệch phân bố missing. Top tương quan: OverallQual 0.79, GrLivArea 0.69, GarageCars 0.64. 31 cột categorical có ít nhất 1 mức hiếm (&lt;10 mẫu).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loại 2 dòng Id=524 và Id=1299 khỏi tập train khi fit mô hình ở P4/P5 (ngoại lai đã biết của dataset, xem FND-0003). Cách điền missing cho nhóm cột 'missing có ý nghĩa' (PoolQC, MiscFeature, Alley, Fence, MasVnrType, FireplaceQu, Garage*, Bsmt*): dùng hằng số 'None' (categorical) hoặc 0 (numeric liên quan), tính từ quyết định FND-0001 - nay xác nhận lại bằng số liệu train thực tế (tỉ lệ khớp audit toàn bộ).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kết luận rút ra từ EDA trên train, theo nguyên tắc chỉ quyết định dựa vào train</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FND-0003,FND-0001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eda_train_summary.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda_train_summary.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tóm tắt EDA trên train + các quyết định rút ra, kèm tham chiếu log</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eda_train.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/eda_train.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Script EDA (chỉ đọc split=='train'), có thể chạy lại độc lập</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1 Kiểm toán dữ liệu (bổ sung)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xem tận mắt 20 dòng ngẫu nhiên trong train (seed=7) theo yêu cầu cổng G1, kiểm tra quan hệ giữa OverallQual/GrLivArea/YearBuilt/GarageCars/SaleCondition với SalePrice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Không phát hiện nhãn bất thường/vô lý: giá tăng hợp lý theo chất lượng, diện tích, năm xây; các dòng SaleCondition='Partial'/'Family' vẫn có giá hợp lý (ngoại trừ 2 điểm đã ghi ở FND-0003, không nằm trong mẫu 20 dòng này). Gate G1 coi như đã đóng đầy đủ (đã có: manifest, missing, trùng lặp ở P1 + xem mẫu bằng mắt ở đây).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cập nhật skill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người dùng cung cấp bản skill dl-project-from-raw-data mới (file .skill upload). Đã thay thế toàn bộ /mnt/skills/plugins/dl-project-from-raw-data bằng bản mới. Thay đổi cốt lõi: quy trình mở rộng từ P0-P9 thành P0-P11, thêm bước P4 'Khám phá dữ liệu (EDA, chỉ trên train)' chính thức (trước đây mình tự đặt tạm là 'P2.5'), và đảo thứ tự: P5 Tiền xử lý giờ đứng TRƯỚC P6 Baseline (trước đây baseline P4 đứng trước tiền xử lý P5). Số hiệu cổng G3(Baseline)/G4(pipeline) giữ nguyên tên nhưng gắn với P6/P7 mới. Đã re-áp dụng lại 2 chỉnh sửa riêng của dự án này (quy ước ghi log tiếng Việt có dấu ở SKILL.md muc 7, log_schema.md, và scripts/log_change.py README_ROWS) vì bản mới người dùng cung cấp không có 2 chỉnh sửa này.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người dùng yêu cầu cập nhật và ghi nhớ skill mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đối chiếu lại tiến độ dự án theo số P mới: P0 Khởi tạo=Done, P1 Kiểm toán=Done, P2 Định nghĩa bài toán=Done, P3 Chia dữ liệu=Done, P4 Khám phá dữ liệu (train)=Done (thực hiện ở các dòng LOG-0020,LOG-0021,FND-0003, lúc đó gắn nhầm nhãn 'P2.5'). Bước tiếp theo chính xác theo skill mới là P5 (Tiền xử lý: dùng scripts/preprocess_tabular.py fit/check), SAU ĐÓ mới tới P6 (Baseline) - đảo lại thứ tự so với thông báo trước đó của mình (đã nói nhầm là 'P4 Baseline' sẽ làm tiếp, nay đính chính lại).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đính chính theo cấu trúc mới của skill, không sửa các dòng log cũ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S-20260925</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cập nhật skill (lần 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người dùng upload lại file skill (cùng tên nhưng nội dung mới hơn bản đã cập nhật trước đó ở LOG-0025/0026). Điểm mới quan trọng: (1) Thêm script scripts/explore_tabular.py chuyên dụng cho P4 - tự tính thang đo, thống kê mô tả, ngoại lai IQR, giá trị ngoài miền hợp lệ, độ lệch phân phối, tương quan, độ liên quan với nhãn (Pearson/ANOVA), tự vẽ biểu đồ vào eda_plots/. (2) scripts/preprocess_tabular.py mở rộng thêm tùy chọn: --valid-range, --drop-missing-thresh, --select-anova-thresh/--select-corr-thresh (chọn đặc trưng), --bin (rời rạc hóa), --pca (giảm chiều). Đã thay thế toàn bộ thư mục skill và re-áp lại 2 chỉnh sửa riêng của dự án (quy ước log tiếng Việt có dấu ở SKILL.md, log_schema.md, log_change.py README_ROWS).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người dùng yêu cầu cập nhật bộ nhớ bằng file skill mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P4 (khám phá dữ liệu) của dự án này đã hoàn thành thủ công trước khi có script explore_tabular.py, kết quả và các DECISION (LOG-0020, LOG-0021, FND-0003) vẫn giữ nguyên giá trị, không cần chạy lại. Ở bước P5 (Tiền xử lý) sắp tới, sẽ tận dụng preprocess_tabular.py bản mới, đặc biệt --valid-range cho các cột có miền giá trị rõ ràng (vd YearBuilt, GarageYrBlt không được lớn hơn năm hiện tại) nếu phù hợp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P4 Khám phá dữ liệu (EDA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">split_v1_selected_features.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01_data/splits/split_v1_selected_features.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tạo bảng con chỉ gồm 67 đặc trưng người dùng chọn lọc theo 9 nhóm ý nghĩa nghiệp vụ (khu đất, vị trí, chất lượng nhà, móng/tầng hầm, hệ thống, diện tích, garage, đường vào, giao dịch) + Id, SalePrice, split. Loại 12 cột: Fireplaces, FireplaceQu, WoodDeckSF, OpenPorchSF, EnclosedPorch, 3SsnPorch, ScreenPorch, PoolArea, PoolQC, Fence, MiscFeature, MiscVal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chạy scripts/explore_tabular.py trên split_v1_selected_features.csv (chỉ train, 1022 dòng, 67 đặc trưng), --label-col SalePrice --label-type numeric --ordinal-cols (17 cột chất lượng/thứ bậc), --valid-range cho LotFrontage/MasVnrArea/GarageYrBlt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28 cột số, 39 cột hạng mục. 0 giá trị ngoài miền hợp lệ. Ngoại lai IQR đáng chú ý: OverallCond 8.41%, MSSubClass 7.24%, LotFrontage 6.95%, MasVnrArea 6.7%, BsmtFinSF2 9.98% (nhưng phần lớn do phân phối lệch/rời rạc, không hẳn là lỗi). Top Pearson-vs-label (numeric, chưa log-transform): OverallQual 0.786, GrLivArea 0.689, TotalBsmtSF 0.592, GarageCars 0.642, GarageArea 0.618, 1stFlrSF 0.583. Heatmap xác nhận 3 cụm cộng tuyến: (GrLivArea, FullBath, TotRmsAbvGrd, 2ndFlrSF), (GarageCars, GarageArea), (TotalBsmtSF, BsmtUnfSF, BsmtFinSF1, 1stFlrSF).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vẽ 9 biểu đồ tổng hợp theo nhóm ý nghĩa nghiệp vụ (N1_KhuDat...N9_GiaoDich), mỗi ô con là scatter(numeric vs SalePrice, có hệ số Pearson) hoặc boxplot(SalePrice theo từng mức categorical, sắp theo median tăng dần). Lưu tại 06_reports/eda/eda_plots/by_group/.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eda_group_plots.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/eda_group_plots.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Script tự viết (bổ sung ngoài skill) để vẽ 9 biểu đồ theo nhóm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theo đề xuất người dùng, chạy explore_tabular.py trên TOÀN BỘ 79 cột gốc (01_data/splits/split_v1.csv, chỉ train) thay vì chỉ 67 cột đã chọn, để đối chiếu ngược và tránh bỏ sót đặc trưng quan trọng.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kết quả 67 cột đã chọn khớp 100% với lần chạy trước. Phát hiện quan trọng ở nhóm 12 cột đã loại: Fireplaces (corr=0.46) và FireplaceQu (eta2=0.302) có tín hiệu MẠNH - cao hơn nhiều cột đang được giữ (vd BldgType eta2=0.048, Electrical eta2=0.079). WoodDeckSF (0.328) và OpenPorchSF (0.315) cũng ở mức trung bình-khá, tương đương HalfBath (0.278) đang được giữ. Ngược lại EnclosedPorch (-0.146), 3SsnPorch (0.062), ScreenPorch (0.143), PoolArea (0.127), MiscVal (-0.015), PoolQC (eta2=0.013), Fence (eta2=0.04), MiscFeature (eta2=0.009) đều xác nhận yếu, loại là hợp lý.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chốt danh sách đặc trưng cuối cùng: 67 cột ban đầu + 4 cột thêm lại (Fireplaces, FireplaceQu vào nhóm 3 - Chất lượng nhà; WoodDeckSF, OpenPorchSF vào nhóm 6 - Diện tích sinh hoạt) = 71 cột. Loại hẳn 8 cột còn lại (EnclosedPorch, 3SsnPorch, ScreenPorch, PoolArea, PoolQC, Fence, MiscFeature, MiscVal) do tín hiệu quá yếu (xem FND-0004).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người dùng đồng ý sau khi xem bằng chứng đối chiếu EDA toàn bộ 79 cột</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FND-0004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MODIFY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cập nhật bảng đặc trưng đã chọn từ 67 lên 71 cột: thêm Fireplaces, FireplaceQu (nhóm 3), WoodDeckSF, OpenPorchSF (nhóm 6) theo DECISION LOG-0034.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chạy lại explore_tabular.py và vẽ lại 2 biểu đồ nhóm (N3, N6) trên bảng 71 cột đã cập nhật.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FireplaceQu cho bậc thang tăng dần rõ theo chất lượng (Po den Ex). WoodDeckSF/OpenPorchSF phân tán nhưng có xu hướng dương rõ. Xác nhận quyết định thêm lại là hợp lý.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">explore_tabular.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/explore_tabular.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copy script explore_tabular.py (từ skill) vào dự án để chạy lại được độc lập, dùng cho cả 06_reports/eda và 06_reports/eda_full</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select_features.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/select_features.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lưu code lọc 71 đặc trưng đã chọn (trước đó chỉ chạy tay, chưa lưu file) thành script chạy lại được: đọc 01_data/splits/split_v1.csv, xuất 01_data/splits/split_v1_selected_features.csv.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chạy lại, so sánh SHA256/MD5 với file hiện có: khớp 100% (6143aaca63ab186570c0c59c30c76f96).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Finding_ID</t>
   </si>
   <si>
@@ -495,6 +708,51 @@
     <t xml:space="preserve">Wontfix</t>
   </si>
   <si>
+    <t xml:space="preserve">FND-0003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ngoại lai / lỗi dữ liệu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01_data/splits/split_v1.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Id=524, Id=1299</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 căn nhà có GrLivArea rất lớn (4676 và 5642 sqft) và OverallQual=10 nhưng SalePrice lại RẤT THẤP (184750 và 160000) - thấp hơn nhiều nhà nhỏ hơn nhiều. Cả 2 đều có SaleCondition='Partial' (nhà bán khi CHƯA hoàn thiện/xây xong). Đây là lỗi/ngoại lai đã được chính tác giả dataset (Dean De Cock) ghi nhận công khai, khuyến nghị loại khỏi tập train. Có 1 điểm thứ 3 (Id=1183, GrLivArea=4476, SalePrice=745000, SaleCondition='Abnorml') là giá cao nhất trong toàn bộ dữ liệu - đây là điểm HỢP LỆ (không phải lỗi), không loại.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02_notebooks/eda_train.png (scatter GrLivArea vs SalePrice); bảng chi tiết 3 dòng GrLivArea&gt;4000 trong train</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECISION: loại 2 dòng Id=524 và Id=1299 khỏi TRAIN khi huấn luyện baseline/mô hình (P4/P5). KHÔNG loại khỏi val/test (val/test không có 2 Id này vì đều rơi vào train ở split_v1, nhưng nguyên tắc chung: ngoại lai chỉ loại ở train). Giữ nguyên Id=1183 vì là giá trị hợp lệ, không phải lỗi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chọn đặc trưng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda_full/eda_report.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trong 12 cột người dùng loại ban đầu (nhóm 'extras'), 3-4 cột thực ra có tín hiệu đáng kể với SalePrice: Fireplaces (corr=0.46), FireplaceQu (eta2=0.302), WoodDeckSF (corr=0.328), OpenPorchSF (corr=0.315). Đây là bằng chứng số liệu (chỉ từ train) nên cân nhắc thêm lại các cột này.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda_full/eda_report.md, mục 'Độ liên quan với biến mục tiêu'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đề xuất: thêm Fireplaces + FireplaceQu (nhóm 3 Chất lượng nhà) và WoodDeckSF + OpenPorchSF (nhóm 6 Diện tích) vào danh sách giữ lại; giữ nguyên loại 8 cột còn lại (EnclosedPorch, 3SsnPorch, ScreenPorch, PoolArea, PoolQC, Fence, MiscFeature, MiscVal). [Đã thực hiện - xem LOG-0034]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FND-0005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã thêm lại 4 cột này vào danh sách giữ (xem LOG tiếp theo).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Loại</t>
   </si>
   <si>
@@ -591,9 +849,6 @@
     <t xml:space="preserve">script kiem toan du lieu (P1)</t>
   </si>
   <si>
-    <t xml:space="preserve">01_data/splits/split_v1.csv</t>
-  </si>
-  <si>
     <t xml:space="preserve">a7efd8bd0070df62801eafc5d8e213858f8ca7d8851dafd4d7115d480b886448</t>
   </si>
   <si>
@@ -618,6 +873,171 @@
     <t xml:space="preserve">định nghĩa bài toán, metric, ràng buộc (P2)</t>
   </si>
   <si>
+    <t xml:space="preserve">02_notebooks/eda_train.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90a6c5317dc2349675bdb1d1801f76467908513c0ad627b7157dbf6bcb603f03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biểu đồ EDA (chỉ train): phân phối SalePrice, GrLivArea vs SalePrice, top tương quan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e45edd39598404486ff8765bedde8eb36d86c3a74629765310d46e6197f24b57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">báo cáo tóm tắt EDA train</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1be7990116f99f9bd87efbf9f313721eb28cb2435ae6838db42cb11808a6bfb2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script EDA (chỉ train)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_report.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0cfd619f752c91e02c96e78d2a4e03fd947661986dcc4e19029d27c4006b05c5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">báo cáo EDA cập nhật trên 71 cột (bản mới nhất, ghi đè bản 67 cột)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7673421343082d3c34fed7dd0fe44f2245431094a129fe4c90c17294ab2477cb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">số liệu EDA dạng máy đọc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_plots/correlation_heatmap.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3f5f9c74b62e31998a215d33b9b0adde52fdfe5afbff94eb932ebc246aa73520</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heatmap tương quan 28 cột số (đại diện cho 30 file trong eda_plots/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_plots/by_group/N1_KhuDat.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0f89df917b99bf9c3b9fbe1637c80e93128857dcdc6d01044655885fe30108b6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biểu đồ quan hệ với SalePrice - nhóm N1_KhuDat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_plots/by_group/N2_ViTri.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">777b6a8d21d058930d17b7dfd0180b2544348f21f87f3108d566ab67fad2711e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biểu đồ quan hệ với SalePrice - nhóm N2_ViTri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_plots/by_group/N3_ChatLuongNha.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f9fb7ea094372d691e63d1523ff4e49cfe8203b401b7d13bb3dc7dd79ff8a818</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cập nhật: thêm Fireplaces/FireplaceQu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_plots/by_group/N4_MongTangHam.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6a4275f39cb430a6a3808f613823a127d183a5f66dc6189fc17c70527dbfee22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biểu đồ quan hệ với SalePrice - nhóm N4_MongTangHam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_plots/by_group/N5_HeThong.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ca55ec7afe0d90692548531b0322c5cfb0da3f021f6f1823d7575d1be72e0651</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biểu đồ quan hệ với SalePrice - nhóm N5_HeThong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_plots/by_group/N6_DienTichSinhHoat.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5f622d6b3107b6ed41e660ed64812557f7f72c1aa90f7cb359999af31d9d96a3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cập nhật: thêm WoodDeckSF/OpenPorchSF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_plots/by_group/N7_Garage.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">852e464147262b85ce9955dc331cf800db60a04e34771e554c8b4cc10db08849</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biểu đồ quan hệ với SalePrice - nhóm N7_Garage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_plots/by_group/N8_DuongVao.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eeef2fce42ca349d7ab57e6ca393a2ecad59248598b7a8d235076967a45de4ef</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biểu đồ quan hệ với SalePrice - nhóm N8_DuongVao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda/eda_plots/by_group/N9_GiaoDich.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c104ff353a9c2eed16eadf17e9094d2dc62891e317e7a95e7c6970ae5c05cfb2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biểu đồ quan hệ với SalePrice - nhóm N9_GiaoDich</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34212d902e49d0fd1db08cdae1e8d5e3f56a856b47f23c3d5423c349070bfa0f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script vẽ biểu đồ EDA theo nhóm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3f5ae97f4b679c7d5896f7a2afc77ebfa423c4fec3b46efce8369df2dbf477ae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">báo cáo EDA đầy đủ 79 cột (đối chiếu với 67 cột đã chọn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/eda_full/eda.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a860a5548eb7324418525edfb8aa365baf8bc3993f362a50d84796e09890dbe1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">số liệu EDA đầy đủ 79 cột</t>
+  </si>
+  <si>
+    <t xml:space="preserve">267a220b2e4b6fc1317a692e78af9c0660fad859de392081f1b9baa54228bf13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script EDA chính thức của skill (P4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7148d38810b4cacfa875b33ff0da4e434e0867392fd3b69d9e06b20923da7065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script lọc 71 đặc trưng đã chọn (P4)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Exp_ID</t>
   </si>
   <si>
@@ -720,15 +1140,9 @@
     <t xml:space="preserve">DISCOVER</t>
   </si>
   <si>
-    <t xml:space="preserve">MODIFY</t>
-  </si>
-  <si>
     <t xml:space="preserve">DELETE</t>
   </si>
   <si>
-    <t xml:space="preserve">VERIFY</t>
-  </si>
-  <si>
     <t xml:space="preserve">Theo trạng thái</t>
   </si>
   <si>
@@ -739,9 +1153,6 @@
   </si>
   <si>
     <t xml:space="preserve">Theo mức độ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High</t>
   </si>
   <si>
     <t xml:space="preserve">Critical</t>
@@ -821,7 +1232,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -832,6 +1243,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
         <bgColor rgb="FF333333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -884,7 +1301,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -930,6 +1347,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -988,7 +1409,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFCE4D6"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -1336,7 +1757,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:X20"/>
+  <dimension ref="A1:X39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
@@ -2381,7 +2802,7 @@
       <c r="W18" s="9"/>
       <c r="X18" s="9"/>
     </row>
-    <row r="19" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
         <v>121</v>
       </c>
@@ -2439,7 +2860,7 @@
       <c r="W19" s="9"/>
       <c r="X19" s="9"/>
     </row>
-    <row r="20" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
         <v>127</v>
       </c>
@@ -2490,6 +2911,1048 @@
       <c r="V20" s="9"/>
       <c r="W20" s="9"/>
       <c r="X20" s="9"/>
+    </row>
+    <row r="21" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>0.688842592592593</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S21" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T21" s="9"/>
+      <c r="U21" s="9"/>
+      <c r="V21" s="9"/>
+      <c r="W21" s="9"/>
+      <c r="X21" s="9" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>0.688854166666667</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I22" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="O22" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="P22" s="9"/>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S22" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T22" s="9"/>
+      <c r="U22" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="V22" s="9"/>
+      <c r="W22" s="9"/>
+      <c r="X22" s="9"/>
+    </row>
+    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>0.689074074074074</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I23" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J23" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="K23" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="L23" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="O23" s="9"/>
+      <c r="P23" s="9"/>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S23" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T23" s="9"/>
+      <c r="U23" s="9"/>
+      <c r="V23" s="9"/>
+      <c r="W23" s="9"/>
+      <c r="X23" s="9"/>
+    </row>
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>0.689074074074074</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="K24" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="L24" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="O24" s="9"/>
+      <c r="P24" s="9"/>
+      <c r="Q24" s="9"/>
+      <c r="R24" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S24" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T24" s="9"/>
+      <c r="U24" s="9"/>
+      <c r="V24" s="9"/>
+      <c r="W24" s="9"/>
+      <c r="X24" s="9"/>
+    </row>
+    <row r="25" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="B25" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C25" s="11" t="n">
+        <v>0.693634259259259</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I25" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="O25" s="9"/>
+      <c r="P25" s="9"/>
+      <c r="Q25" s="9"/>
+      <c r="R25" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S25" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T25" s="9"/>
+      <c r="U25" s="9"/>
+      <c r="V25" s="9"/>
+      <c r="W25" s="9"/>
+      <c r="X25" s="9" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="B26" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C26" s="11" t="n">
+        <v>0.969212962962963</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="O26" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="P26" s="9"/>
+      <c r="Q26" s="9"/>
+      <c r="R26" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S26" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T26" s="9"/>
+      <c r="U26" s="9"/>
+      <c r="V26" s="9"/>
+      <c r="W26" s="9"/>
+      <c r="X26" s="9"/>
+    </row>
+    <row r="27" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B27" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>0.969212962962963</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I27" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="J27" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="O27" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="P27" s="9"/>
+      <c r="Q27" s="9"/>
+      <c r="R27" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S27" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T27" s="9"/>
+      <c r="U27" s="9"/>
+      <c r="V27" s="9"/>
+      <c r="W27" s="9"/>
+      <c r="X27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="B28" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>0.580555555555556</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="J28" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
+      <c r="M28" s="9"/>
+      <c r="N28" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="O28" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="P28" s="9"/>
+      <c r="Q28" s="9"/>
+      <c r="R28" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S28" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T28" s="9"/>
+      <c r="U28" s="9"/>
+      <c r="V28" s="9"/>
+      <c r="W28" s="9"/>
+      <c r="X28" s="9"/>
+    </row>
+    <row r="29" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="B29" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C29" s="11" t="n">
+        <v>0.580555555555556</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I29" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="J29" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="K29" s="9"/>
+      <c r="L29" s="9"/>
+      <c r="M29" s="9"/>
+      <c r="N29" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="O29" s="9"/>
+      <c r="P29" s="9"/>
+      <c r="Q29" s="9"/>
+      <c r="R29" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S29" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T29" s="9"/>
+      <c r="U29" s="9"/>
+      <c r="V29" s="9"/>
+      <c r="W29" s="9"/>
+      <c r="X29" s="9"/>
+    </row>
+    <row r="30" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>0.598553240740741</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I30" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J30" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K30" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="L30" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="M30" s="9"/>
+      <c r="N30" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="O30" s="9"/>
+      <c r="P30" s="9"/>
+      <c r="Q30" s="9"/>
+      <c r="R30" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S30" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T30" s="9"/>
+      <c r="U30" s="9"/>
+      <c r="V30" s="9"/>
+      <c r="W30" s="9"/>
+      <c r="X30" s="9"/>
+    </row>
+    <row r="31" customFormat="false" ht="168.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B31" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C31" s="11" t="n">
+        <v>0.598564814814815</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I31" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="J31" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K31" s="9"/>
+      <c r="L31" s="9"/>
+      <c r="M31" s="9"/>
+      <c r="N31" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="O31" s="9"/>
+      <c r="P31" s="9"/>
+      <c r="Q31" s="9"/>
+      <c r="R31" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S31" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T31" s="9"/>
+      <c r="U31" s="9"/>
+      <c r="V31" s="9"/>
+      <c r="W31" s="9"/>
+      <c r="X31" s="9" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C32" s="11" t="n">
+        <v>0.602893518518519</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I32" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J32" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K32" s="9"/>
+      <c r="L32" s="9"/>
+      <c r="M32" s="9"/>
+      <c r="N32" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="O32" s="9"/>
+      <c r="P32" s="9"/>
+      <c r="Q32" s="9"/>
+      <c r="R32" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S32" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T32" s="9"/>
+      <c r="U32" s="9"/>
+      <c r="V32" s="9"/>
+      <c r="W32" s="9"/>
+      <c r="X32" s="9"/>
+    </row>
+    <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B33" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>0.602951388888889</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H33" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I33" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J33" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K33" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="L33" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S33" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T33" s="9"/>
+      <c r="U33" s="9"/>
+      <c r="V33" s="9"/>
+      <c r="W33" s="9"/>
+      <c r="X33" s="9"/>
+    </row>
+    <row r="34" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>0.618171296296296</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H34" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I34" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="J34" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S34" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T34" s="9"/>
+      <c r="U34" s="9"/>
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B35" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>0.619652777777778</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I35" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="J35" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="O35" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S35" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+    </row>
+    <row r="36" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B36" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>0.78525462962963</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H36" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I36" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J36" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K36" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="L36" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S36" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+    </row>
+    <row r="37" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="B37" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>0.78525462962963</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H37" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I37" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="J37" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K37" s="9"/>
+      <c r="L37" s="9"/>
+      <c r="M37" s="9"/>
+      <c r="N37" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="O37" s="9"/>
+      <c r="P37" s="9"/>
+      <c r="Q37" s="9"/>
+      <c r="R37" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S37" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T37" s="9"/>
+      <c r="U37" s="9"/>
+      <c r="V37" s="9"/>
+      <c r="W37" s="9"/>
+      <c r="X37" s="9" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="B38" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>0.788993055555556</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G38" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H38" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I38" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J38" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K38" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="L38" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="M38" s="9"/>
+      <c r="N38" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="O38" s="9"/>
+      <c r="P38" s="9"/>
+      <c r="Q38" s="9"/>
+      <c r="R38" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S38" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T38" s="9"/>
+      <c r="U38" s="9"/>
+      <c r="V38" s="9"/>
+      <c r="W38" s="9"/>
+      <c r="X38" s="9"/>
+    </row>
+    <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="B39" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>0.792743055555556</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H39" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I39" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J39" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="K39" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="L39" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="M39" s="9"/>
+      <c r="N39" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="O39" s="9"/>
+      <c r="P39" s="9"/>
+      <c r="Q39" s="9"/>
+      <c r="R39" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S39" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T39" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="U39" s="9"/>
+      <c r="V39" s="9"/>
+      <c r="W39" s="9"/>
+      <c r="X39" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:X1"/>
@@ -2527,7 +3990,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -2546,16 +4009,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>130</v>
+        <v>201</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>131</v>
+        <v>202</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>132</v>
+        <v>203</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>26</v>
@@ -2564,91 +4027,195 @@
         <v>27</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>133</v>
+        <v>204</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>134</v>
+        <v>205</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>135</v>
+        <v>206</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>136</v>
+        <v>207</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>11</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>137</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>138</v>
+        <v>209</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46288</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>139</v>
+        <v>210</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>140</v>
+        <v>211</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>93</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>141</v>
+        <v>212</v>
       </c>
       <c r="G2" s="6"/>
       <c r="H2" s="6" t="s">
-        <v>142</v>
+        <v>213</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>143</v>
+        <v>214</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>144</v>
+        <v>215</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>145</v>
+        <v>216</v>
       </c>
       <c r="L2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>146</v>
+        <v>217</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>46289</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>147</v>
+        <v>218</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>148</v>
+        <v>219</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>114</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>149</v>
+        <v>220</v>
       </c>
       <c r="G3" s="9"/>
       <c r="H3" s="9" t="s">
-        <v>150</v>
+        <v>221</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>151</v>
+        <v>222</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>152</v>
+        <v>223</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>153</v>
+        <v>224</v>
       </c>
       <c r="L3" s="9"/>
+    </row>
+    <row r="4" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="L4" s="9"/>
+    </row>
+    <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="L5" s="9"/>
+    </row>
+    <row r="6" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="K6" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="L6" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
@@ -2678,7 +4245,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="56"/>
@@ -2694,39 +4261,39 @@
         <v>28</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>154</v>
+        <v>240</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>155</v>
+        <v>241</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>156</v>
+        <v>242</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>157</v>
+        <v>243</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>158</v>
+        <v>244</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>159</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>141</v>
+        <v>212</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>160</v>
+        <v>246</v>
       </c>
       <c r="C2" s="6" t="n">
         <v>460676</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>161</v>
+        <v>247</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>162</v>
+        <v>248</v>
       </c>
       <c r="F2" s="7" t="n">
         <v>46287</v>
@@ -2738,16 +4305,16 @@
         <v>72</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>163</v>
+        <v>249</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>365</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>164</v>
+        <v>250</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>165</v>
+        <v>251</v>
       </c>
       <c r="F3" s="7" t="n">
         <v>46287</v>
@@ -2759,16 +4326,16 @@
         <v>76</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>166</v>
+        <v>252</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>415</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>167</v>
+        <v>253</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>168</v>
+        <v>254</v>
       </c>
       <c r="F4" s="7" t="n">
         <v>46287</v>
@@ -2780,16 +4347,16 @@
         <v>80</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>169</v>
+        <v>255</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>420</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>170</v>
+        <v>256</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>171</v>
+        <v>257</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>46287</v>
@@ -2798,19 +4365,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>172</v>
+        <v>258</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>160</v>
+        <v>246</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>192</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>173</v>
+        <v>259</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>174</v>
+        <v>260</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>46288</v>
@@ -2819,19 +4386,19 @@
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>175</v>
+        <v>261</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>176</v>
+        <v>262</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>22802</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>177</v>
+        <v>263</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>178</v>
+        <v>264</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>46288</v>
@@ -2840,19 +4407,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>179</v>
+        <v>265</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>180</v>
+        <v>266</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>9524</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>181</v>
+        <v>267</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>182</v>
+        <v>268</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>46288</v>
@@ -2864,16 +4431,16 @@
         <v>98</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>183</v>
+        <v>269</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>13590</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>184</v>
+        <v>270</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>185</v>
+        <v>271</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>46288</v>
@@ -2882,19 +4449,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>186</v>
+        <v>228</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>160</v>
+        <v>246</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>468785</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>187</v>
+        <v>272</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>188</v>
+        <v>273</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>46289</v>
@@ -2903,19 +4470,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>149</v>
+        <v>220</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>176</v>
+        <v>262</v>
       </c>
       <c r="C11" s="9" t="n">
         <v>48765</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>189</v>
+        <v>274</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>190</v>
+        <v>275</v>
       </c>
       <c r="F11" s="10" t="n">
         <v>46289</v>
@@ -2927,42 +4494,462 @@
         <v>119</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>183</v>
+        <v>269</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>9337</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>191</v>
+        <v>276</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>192</v>
+        <v>277</v>
       </c>
       <c r="F12" s="10" t="n">
         <v>46289</v>
       </c>
       <c r="G12" s="9"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
         <v>124</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>180</v>
+        <v>266</v>
       </c>
       <c r="C13" s="9" t="n">
         <v>2868</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>193</v>
+        <v>278</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>194</v>
+        <v>279</v>
       </c>
       <c r="F13" s="10" t="n">
         <v>46289</v>
       </c>
       <c r="G13" s="9"/>
+    </row>
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>141791</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="G14" s="9"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>1416</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>2595</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>46289</v>
+      </c>
+      <c r="G16" s="9"/>
+    </row>
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>18407</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>51730</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G18" s="9"/>
+    </row>
+    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>150866</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>227085</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="F20" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G20" s="9"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>300</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>70321</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="F21" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>440073</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="F22" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G22" s="9"/>
+    </row>
+    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>263530</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>308</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="s">
+        <v>309</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>63054</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>310</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="F24" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G24" s="9"/>
+    </row>
+    <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="s">
+        <v>312</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>373125</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>202395</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G26" s="9"/>
+    </row>
+    <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>17992</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>320</v>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
+        <v>321</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>108430</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>323</v>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G28" s="9"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>2667</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>325</v>
+      </c>
+      <c r="F29" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>19801</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>326</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>327</v>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G30" s="9"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>70580</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="F31" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>13093</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>331</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>332</v>
+      </c>
+      <c r="F32" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G32" s="9"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>2580</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="F33" s="10" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G33" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
@@ -3016,88 +5003,88 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>195</v>
+        <v>335</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>131</v>
+        <v>202</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>196</v>
+        <v>336</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>197</v>
+        <v>337</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>198</v>
+        <v>338</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>199</v>
+        <v>339</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>200</v>
+        <v>340</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>201</v>
+        <v>341</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>202</v>
+        <v>342</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>203</v>
+        <v>343</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>204</v>
+        <v>344</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>205</v>
+        <v>345</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>206</v>
+        <v>346</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>207</v>
+        <v>347</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>208</v>
+        <v>348</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>209</v>
+        <v>349</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>210</v>
+        <v>350</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>211</v>
+        <v>351</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>212</v>
+        <v>352</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>213</v>
+        <v>353</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>214</v>
+        <v>354</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>215</v>
+        <v>355</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>216</v>
+        <v>356</v>
       </c>
       <c r="Y1" s="5" t="s">
-        <v>217</v>
+        <v>357</v>
       </c>
       <c r="Z1" s="5" t="s">
-        <v>218</v>
+        <v>358</v>
       </c>
       <c r="AA1" s="5" t="s">
         <v>11</v>
       </c>
       <c r="AB1" s="5" t="s">
-        <v>137</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -3134,358 +5121,358 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
+        <v>359</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
-        <v>220</v>
-      </c>
-      <c r="B3" s="12" t="n">
+      <c r="A3" s="13" t="s">
+        <v>360</v>
+      </c>
+      <c r="B3" s="13" t="n">
         <f aca="false">COUNTA(Change_Log!A2:A5000)</f>
-        <v>19</v>
-      </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12" t="s">
-        <v>221</v>
-      </c>
-      <c r="E3" s="12" t="n">
+        <v>38</v>
+      </c>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13" t="s">
+        <v>361</v>
+      </c>
+      <c r="E3" s="13" t="n">
         <f aca="false">COUNTA(Experiments!A2:A5000)</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
-        <v>222</v>
-      </c>
-      <c r="B4" s="12" t="n">
+      <c r="A4" s="13" t="s">
+        <v>362</v>
+      </c>
+      <c r="B4" s="13" t="n">
         <f aca="false">COUNTA(Findings!A2:A5000)</f>
-        <v>2</v>
-      </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12" t="s">
-        <v>223</v>
-      </c>
-      <c r="E4" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13" t="s">
+        <v>363</v>
+      </c>
+      <c r="E4" s="13" t="n">
         <f aca="false">COUNTIF(Experiments!AA2:AA5000,"Done")</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="B5" s="12" t="n">
+      <c r="A5" s="13" t="s">
+        <v>364</v>
+      </c>
+      <c r="B5" s="13" t="n">
         <f aca="false">COUNTIF(Findings!K2:K5000,"Open")</f>
-        <v>1</v>
-      </c>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12" t="s">
-        <v>225</v>
-      </c>
-      <c r="E5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13" t="s">
+        <v>365</v>
+      </c>
+      <c r="E5" s="13" t="n">
         <f aca="false">COUNTIF(Experiments!AA2:AA5000,"Failed")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
+      <c r="A7" s="14" t="s">
+        <v>366</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
-        <v>227</v>
-      </c>
-      <c r="B8" s="12" t="n">
+      <c r="A8" s="13" t="s">
+        <v>367</v>
+      </c>
+      <c r="B8" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A8)</f>
         <v>0</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="B9" s="12" t="n">
+      <c r="A9" s="13" t="s">
+        <v>368</v>
+      </c>
+      <c r="B9" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A9)</f>
         <v>0</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A10)</f>
-        <v>8</v>
-      </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
+        <v>15</v>
+      </c>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>229</v>
-      </c>
-      <c r="B11" s="12" t="n">
+      <c r="A11" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="B11" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A11)</f>
-        <v>0</v>
-      </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A12)</f>
         <v>4</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>230</v>
-      </c>
-      <c r="B13" s="12" t="n">
+      <c r="A13" s="13" t="s">
+        <v>369</v>
+      </c>
+      <c r="B13" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A13)</f>
         <v>0</v>
       </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A14)</f>
-        <v>2</v>
-      </c>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
+        <v>6</v>
+      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="B15" s="12" t="n">
+      <c r="A15" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="B15" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A15)</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
+        <v>1</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A16)</f>
-        <v>4</v>
-      </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
+        <v>6</v>
+      </c>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B17" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A17)</f>
-        <v>1</v>
-      </c>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
+        <v>5</v>
+      </c>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
+      <c r="A19" s="14" t="s">
+        <v>370</v>
+      </c>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B20" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!S2:S5000,A20)</f>
-        <v>19</v>
-      </c>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
+        <v>38</v>
+      </c>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="B21" s="12" t="n">
+      <c r="A21" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="B21" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!S2:S5000,A21)</f>
         <v>0</v>
       </c>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
-        <v>233</v>
-      </c>
-      <c r="B22" s="12" t="n">
+      <c r="A22" s="13" t="s">
+        <v>371</v>
+      </c>
+      <c r="B22" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!S2:S5000,A22)</f>
         <v>0</v>
       </c>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="B23" s="12" t="n">
+      <c r="A23" s="13" t="s">
+        <v>372</v>
+      </c>
+      <c r="B23" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!S2:S5000,A23)</f>
         <v>0</v>
       </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="B24" s="12" t="n">
+      <c r="A24" s="13" t="s">
+        <v>224</v>
+      </c>
+      <c r="B24" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!S2:S5000,A24)</f>
         <v>0</v>
       </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
-        <v>235</v>
-      </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
+      <c r="A26" s="14" t="s">
+        <v>373</v>
+      </c>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="12" t="n">
+      <c r="B27" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!R2:R5000,A27)</f>
-        <v>19</v>
-      </c>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
+        <v>38</v>
+      </c>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="B28" s="12" t="n">
+      <c r="A28" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="B28" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!R2:R5000,A28)</f>
         <v>0</v>
       </c>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="B29" s="12" t="n">
+      <c r="A29" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="B29" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!R2:R5000,A29)</f>
         <v>0</v>
       </c>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12" t="s">
-        <v>236</v>
-      </c>
-      <c r="B30" s="12" t="n">
+      <c r="A30" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="B30" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!R2:R5000,A30)</f>
         <v>0</v>
       </c>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12" t="s">
-        <v>237</v>
-      </c>
-      <c r="B31" s="12" t="n">
+      <c r="A31" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="B31" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!R2:R5000,A31)</f>
         <v>0</v>
       </c>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
tiền xử lý dữ liệu
</commit_message>
<xml_diff>
--- a/house_price_ml/07_logs/change_log.xlsx
+++ b/house_price_ml/07_logs/change_log.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="474">
   <si>
     <t xml:space="preserve">change_log.xlsx - Nhật ký thay đổi dự án ML</t>
   </si>
@@ -636,6 +636,189 @@
     <t xml:space="preserve">Chạy lại, so sánh SHA256/MD5 với file hiện có: khớp 100% (6143aaca63ab186570c0c59c30c76f96).</t>
   </si>
   <si>
+    <t xml:space="preserve">LOG-0039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S-20260926</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P5 Tiền xử lý</t>
+  </si>
+  <si>
+    <t xml:space="preserve">encode_business_rules.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/encode_business_rules.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Script áp quy tắc nghiệp vụ cố định (không học từ dữ liệu, áp đồng nhất train/val/test): mã hóa Ordinal cho 18 cột chất lượng/thứ bậc theo đúng thứ tự (NA=hạng 0 cho cột có thể 'không có đặc điểm'); điền 0 cho MasVnrArea, GarageYrBlt khi thiếu (missing có ý nghĩa, FND-0001); loại 2 dòng ngoại lai Id=524,1299 (FND-0003).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chạy encode_business_rules.py rồi preprocess_tabular.py fit trên 01_data/splits/split_v1_prepped.csv (--label-col SalePrice --impute median --scaler standard --valid-range LotFrontage:0:None --dedup-train).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kết quả: 1020 dòng train (loại 0 trùng), 219 val, 219 test. 49 cột số + 22 cột hạng mục (đúng = 71 - 18 ordinal đã thành số). Tổng sau one-hot: 205 đặc trưng. LotFrontage: 0 giá trị ngoài miền. Cảnh báo (không phải lỗi): val/test có vài mức hạng mục hiếm chưa xuất hiện ở train (RoofMatl='Roll', Exterior1st='Stone', Electrical='Mix') -&gt; tự động mã hóa thành vector 0 (handle_unknown='ignore'), đúng hành vi mong đợi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chạy preprocess_tabular.py check để xác nhận bộ tiền xử lý chỉ học từ train, không rò rỉ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kết quả: KIỂM CHỨNG: PASSED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preprocess_tabular.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/preprocess_tabular.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copy script preprocess_tabular.py (từ skill) vào dự án - script này đã tạo ra thư mục 01_data/processed/ ở bước P5, chạy lại được độc lập</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rà soát quy tắc copy script</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scaffold_project.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/scaffold_project.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rà soát lại toàn bộ project theo quy tắc mới (mọi file do script tạo ra phải có script kèm theo), phát hiện thiếu scaffold_project.py (đã tạo cấu trúc thư mục, README.md, requirements.txt, change_log.xlsx ban đầu ở P0) và log_change.py (đã tạo/ghi toàn bộ change_log.xlsx từ đầu tới giờ). Copy bù cả 2 vào 03_src/scripts/.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_change.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/log_change.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copy bù log_change.py (script tạo/ghi toàn bộ change_log.xlsx)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sắp xếp lại 03_src/scripts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di chuyển vào thư mục 'chung' vì dùng xuyên suốt mọi bước, không riêng bước nào</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/chung/log_change.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di chuyển vào thư mục p0_khoi_tao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/p0_khoi_tao/scaffold_project.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di chuyển vào thư mục p1_kiem_toan_du_lieu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/p1_kiem_toan_du_lieu/audit_dataset.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di chuyển vào thư mục p3_chia_du_lieu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/p3_chia_du_lieu/make_splits.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di chuyển vào thư mục p4_kham_pha_du_lieu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/p4_kham_pha_du_lieu/eda_train.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/p4_kham_pha_du_lieu/select_features.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/p4_kham_pha_du_lieu/explore_tabular.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/p4_kham_pha_du_lieu/eda_group_plots.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di chuyển vào thư mục p5_tien_xu_ly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/p5_tien_xu_ly/encode_business_rules.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03_src/scripts/p5_tien_xu_ly/preprocess_tabular.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thêm sơ đồ cấu trúc 03_src/scripts/ mới (theo bước) vào README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sửa script tự tạo thư mục 06_reports/eda/eda_plots/by_group/ bằng os.makedirs(exist_ok=True), không cần mkdir tay trước khi chạy nữa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOG-0057</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quy_trinh_chay_lai.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06_reports/quy_trinh_chay_lai.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tạo/cập nhật tài liệu quy trình chạy lại toàn bộ pipeline (người dùng cung cấp bản nháp, mình cập nhật đường dẫn theo cấu trúc thư mục mới, hoàn thiện Bước 8/9 còn thiếu tiêu đề, thêm Bước 10 (kiểm chứng check) còn thiếu).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Finding_ID</t>
   </si>
   <si>
@@ -1036,6 +1219,120 @@
   </si>
   <si>
     <t xml:space="preserve">script lọc 71 đặc trưng đã chọn (P4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01_data/splits/split_v1_prepped.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">423b3d8395fd06c51a182b039182e78e84c006d513c61fddaf2cdefa4a3b3a8a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bảng 71 đặc trưng sau khi áp quy tắc nghiệp vụ (trước preprocess_tabular.py)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01_data/processed/preprocessor.joblib</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joblib</t>
+  </si>
+  <si>
+    <t xml:space="preserve">62f7355e882d8c24c83b1c9e3f2fe5b036cf08db361ebd754ceb08da453a27bc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bộ tiền xử lý đã fit (impute+scale+onehot), dùng để apply cho dữ liệu mới sau này</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01_data/processed/preprocess_meta.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c9fe12b871e87f210f2f3e53fcc6f3ca0d0e12e6e001241b5c0eaf4eef8ddf29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metadata: danh sách cột, tham số impute/scale đã học</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01_data/processed/processed_train.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cc5da2c468bf3986f67b24e65ab0ca0ed4c6166c5b4cc4b605d9c912acc330eb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dữ liệu train đã tiền xử lý (1020 dòng x 205 đặc trưng)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01_data/processed/processed_val.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11ff797cd5a7885455f0ee595da251a8a0f604063e3a0570ff20c0a64931c2a6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dữ liệu val đã tiền xử lý</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01_data/processed/processed_test.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">274673333c44f596da90075d477a8de16ae59e29c259be6bd4e40050825a4740</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dữ liệu test đã tiền xử lý (chưa mở, chỉ dùng ở đánh giá cuối)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">183bbc29009277c54b30266eae37b5c3f8d5469a906f90b70b19363deb82d517</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script tiền xử lý chính thức của skill (P5), fit/check/apply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8256c29b9f6310fa477352621dd19822a1e35ee57f10c02a2a7651b6a5bb121d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script khởi tạo cấu trúc project (P0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b454e4193e94852ed3ea5a03345ef36bb829eb20f848904fbc15458d9986653e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script ghi change_log.xlsx (dùng xuyên suốt mọi bước)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script ghi change_log.xlsx (dùng xuyên suốt mọi bước) - đường dẫn mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script khởi tạo cấu trúc project (P0) - đường dẫn mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script kiểm toán dữ liệu (P1) - đường dẫn mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script chia train/val/test (P3) - đường dẫn mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script EDA thủ công ban đầu (P4) - đường dẫn mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script lọc 71 đặc trưng đã chọn (P4) - đường dẫn mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script EDA chính thức của skill (P4) - đường dẫn mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script vẽ biểu đồ EDA theo nhóm (P4) - đường dẫn mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bf4418ca18dd95b1a0a4c92e127e31851a9521a7285fe3381b3bdcc7fd493009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script áp quy tắc nghiệp vụ cố định (P5) - đường dẫn mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">script tiền xử lý chính thức của skill (P5) - đường dẫn mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10e12473d54c3046f7276b453c47a6aaf2e7e0affb1d9c7b779190211b7cde6d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">runbook: toàn bộ lệnh chạy lại pipeline P0-P5</t>
   </si>
   <si>
     <t xml:space="preserve">Exp_ID</t>
@@ -1757,7 +2054,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:X39"/>
+  <dimension ref="A1:X58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
@@ -3896,7 +4193,7 @@
       <c r="W38" s="9"/>
       <c r="X38" s="9"/>
     </row>
-    <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
         <v>196</v>
       </c>
@@ -3953,6 +4250,1086 @@
       <c r="V39" s="9"/>
       <c r="W39" s="9"/>
       <c r="X39" s="9"/>
+    </row>
+    <row r="40" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="B40" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C40" s="11" t="n">
+        <v>0.390138888888889</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F40" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G40" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H40" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I40" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J40" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="K40" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="L40" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="M40" s="9"/>
+      <c r="N40" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="O40" s="9"/>
+      <c r="P40" s="9"/>
+      <c r="Q40" s="9"/>
+      <c r="R40" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S40" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T40" s="9"/>
+      <c r="U40" s="9"/>
+      <c r="V40" s="9"/>
+      <c r="W40" s="9"/>
+      <c r="X40" s="9"/>
+    </row>
+    <row r="41" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B41" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>0.390150462962963</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H41" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I41" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="J41" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="K41" s="9"/>
+      <c r="L41" s="9"/>
+      <c r="M41" s="9"/>
+      <c r="N41" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="O41" s="9"/>
+      <c r="P41" s="9"/>
+      <c r="Q41" s="9"/>
+      <c r="R41" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S41" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T41" s="9"/>
+      <c r="U41" s="9"/>
+      <c r="V41" s="9"/>
+      <c r="W41" s="9"/>
+      <c r="X41" s="9" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B42" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C42" s="11" t="n">
+        <v>0.390150462962963</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H42" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I42" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="J42" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="K42" s="9"/>
+      <c r="L42" s="9"/>
+      <c r="M42" s="9"/>
+      <c r="N42" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="O42" s="9"/>
+      <c r="P42" s="9"/>
+      <c r="Q42" s="9"/>
+      <c r="R42" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S42" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T42" s="9"/>
+      <c r="U42" s="9"/>
+      <c r="V42" s="9"/>
+      <c r="W42" s="9"/>
+      <c r="X42" s="9" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="B43" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>0.414710648148148</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I43" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J43" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="K43" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="L43" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="M43" s="9"/>
+      <c r="N43" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="O43" s="9"/>
+      <c r="P43" s="9"/>
+      <c r="Q43" s="9"/>
+      <c r="R43" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S43" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T43" s="9"/>
+      <c r="U43" s="9"/>
+      <c r="V43" s="9"/>
+      <c r="W43" s="9"/>
+      <c r="X43" s="9"/>
+    </row>
+    <row r="44" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C44" s="11" t="n">
+        <v>0.415752314814815</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G44" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H44" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I44" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J44" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="K44" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="L44" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="M44" s="9"/>
+      <c r="N44" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="O44" s="9"/>
+      <c r="P44" s="9"/>
+      <c r="Q44" s="9"/>
+      <c r="R44" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S44" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T44" s="9"/>
+      <c r="U44" s="9"/>
+      <c r="V44" s="9"/>
+      <c r="W44" s="9"/>
+      <c r="X44" s="9"/>
+    </row>
+    <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="B45" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C45" s="11" t="n">
+        <v>0.415763888888889</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H45" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I45" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J45" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="K45" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="L45" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="M45" s="9"/>
+      <c r="N45" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="O45" s="9"/>
+      <c r="P45" s="9"/>
+      <c r="Q45" s="9"/>
+      <c r="R45" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S45" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T45" s="9"/>
+      <c r="U45" s="9"/>
+      <c r="V45" s="9"/>
+      <c r="W45" s="9"/>
+      <c r="X45" s="9"/>
+    </row>
+    <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="B46" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C46" s="11" t="n">
+        <v>0.435486111111111</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G46" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H46" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I46" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J46" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K46" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="L46" s="9"/>
+      <c r="M46" s="9"/>
+      <c r="N46" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="O46" s="9"/>
+      <c r="P46" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="Q46" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="R46" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S46" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T46" s="9"/>
+      <c r="U46" s="9"/>
+      <c r="V46" s="9"/>
+      <c r="W46" s="9"/>
+      <c r="X46" s="9"/>
+    </row>
+    <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B47" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C47" s="11" t="n">
+        <v>0.435486111111111</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H47" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I47" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J47" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K47" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="L47" s="9"/>
+      <c r="M47" s="9"/>
+      <c r="N47" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="O47" s="9"/>
+      <c r="P47" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="Q47" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="R47" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S47" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T47" s="9"/>
+      <c r="U47" s="9"/>
+      <c r="V47" s="9"/>
+      <c r="W47" s="9"/>
+      <c r="X47" s="9"/>
+    </row>
+    <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="B48" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>0.435486111111111</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F48" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H48" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I48" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J48" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K48" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="L48" s="9"/>
+      <c r="M48" s="9"/>
+      <c r="N48" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="O48" s="9"/>
+      <c r="P48" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q48" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="R48" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S48" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T48" s="9"/>
+      <c r="U48" s="9"/>
+      <c r="V48" s="9"/>
+      <c r="W48" s="9"/>
+      <c r="X48" s="9"/>
+    </row>
+    <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="B49" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C49" s="11" t="n">
+        <v>0.435486111111111</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F49" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H49" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I49" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J49" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K49" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="L49" s="9"/>
+      <c r="M49" s="9"/>
+      <c r="N49" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="O49" s="9"/>
+      <c r="P49" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q49" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="R49" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S49" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T49" s="9"/>
+      <c r="U49" s="9"/>
+      <c r="V49" s="9"/>
+      <c r="W49" s="9"/>
+      <c r="X49" s="9"/>
+    </row>
+    <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="B50" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C50" s="11" t="n">
+        <v>0.435486111111111</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H50" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I50" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J50" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K50" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="L50" s="9"/>
+      <c r="M50" s="9"/>
+      <c r="N50" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="O50" s="9"/>
+      <c r="P50" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q50" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="R50" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S50" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T50" s="9"/>
+      <c r="U50" s="9"/>
+      <c r="V50" s="9"/>
+      <c r="W50" s="9"/>
+      <c r="X50" s="9"/>
+    </row>
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="B51" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C51" s="11" t="n">
+        <v>0.435486111111111</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H51" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I51" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J51" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K51" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="L51" s="9"/>
+      <c r="M51" s="9"/>
+      <c r="N51" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="O51" s="9"/>
+      <c r="P51" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q51" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="R51" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S51" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T51" s="9"/>
+      <c r="U51" s="9"/>
+      <c r="V51" s="9"/>
+      <c r="W51" s="9"/>
+      <c r="X51" s="9"/>
+    </row>
+    <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="B52" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>0.435486111111111</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H52" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I52" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J52" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K52" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="L52" s="9"/>
+      <c r="M52" s="9"/>
+      <c r="N52" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="O52" s="9"/>
+      <c r="P52" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q52" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="R52" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S52" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T52" s="9"/>
+      <c r="U52" s="9"/>
+      <c r="V52" s="9"/>
+      <c r="W52" s="9"/>
+      <c r="X52" s="9"/>
+    </row>
+    <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="B53" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C53" s="11" t="n">
+        <v>0.435486111111111</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H53" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I53" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J53" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K53" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="L53" s="9"/>
+      <c r="M53" s="9"/>
+      <c r="N53" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="O53" s="9"/>
+      <c r="P53" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q53" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="R53" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S53" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T53" s="9"/>
+      <c r="U53" s="9"/>
+      <c r="V53" s="9"/>
+      <c r="W53" s="9"/>
+      <c r="X53" s="9"/>
+    </row>
+    <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="B54" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C54" s="11" t="n">
+        <v>0.435486111111111</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E54" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F54" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H54" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I54" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J54" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K54" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="L54" s="9"/>
+      <c r="M54" s="9"/>
+      <c r="N54" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="O54" s="9"/>
+      <c r="P54" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q54" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="R54" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S54" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T54" s="9"/>
+      <c r="U54" s="9"/>
+      <c r="V54" s="9"/>
+      <c r="W54" s="9"/>
+      <c r="X54" s="9"/>
+    </row>
+    <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="B55" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C55" s="11" t="n">
+        <v>0.435486111111111</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H55" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I55" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J55" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K55" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="L55" s="9"/>
+      <c r="M55" s="9"/>
+      <c r="N55" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="O55" s="9"/>
+      <c r="P55" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q55" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="R55" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S55" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T55" s="9"/>
+      <c r="U55" s="9"/>
+      <c r="V55" s="9"/>
+      <c r="W55" s="9"/>
+      <c r="X55" s="9"/>
+    </row>
+    <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="B56" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C56" s="11" t="n">
+        <v>0.435763888888889</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E56" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H56" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I56" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="J56" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K56" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="L56" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="M56" s="9"/>
+      <c r="N56" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="O56" s="9"/>
+      <c r="P56" s="9"/>
+      <c r="Q56" s="9"/>
+      <c r="R56" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S56" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T56" s="9"/>
+      <c r="U56" s="9"/>
+      <c r="V56" s="9"/>
+      <c r="W56" s="9"/>
+      <c r="X56" s="9"/>
+    </row>
+    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="B57" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C57" s="11" t="n">
+        <v>0.437268518518519</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H57" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I57" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="J57" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K57" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="L57" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="M57" s="9"/>
+      <c r="N57" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="O57" s="9"/>
+      <c r="P57" s="9"/>
+      <c r="Q57" s="9"/>
+      <c r="R57" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S57" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T57" s="9"/>
+      <c r="U57" s="9"/>
+      <c r="V57" s="9"/>
+      <c r="W57" s="9"/>
+      <c r="X57" s="9"/>
+    </row>
+    <row r="58" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="B58" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C58" s="11" t="n">
+        <v>0.437268518518519</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G58" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H58" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="I58" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J58" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="K58" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="L58" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="M58" s="9"/>
+      <c r="N58" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="O58" s="9"/>
+      <c r="P58" s="9"/>
+      <c r="Q58" s="9"/>
+      <c r="R58" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S58" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="T58" s="9"/>
+      <c r="U58" s="9"/>
+      <c r="V58" s="9"/>
+      <c r="W58" s="9"/>
+      <c r="X58" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:X1"/>
@@ -4009,16 +5386,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>201</v>
+        <v>262</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>202</v>
+        <v>263</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>203</v>
+        <v>264</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>26</v>
@@ -4027,125 +5404,125 @@
         <v>27</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>204</v>
+        <v>265</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>205</v>
+        <v>266</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>206</v>
+        <v>267</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>207</v>
+        <v>268</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>11</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>208</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>209</v>
+        <v>270</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>46288</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>210</v>
+        <v>271</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>211</v>
+        <v>272</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>93</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>212</v>
+        <v>273</v>
       </c>
       <c r="G2" s="6"/>
       <c r="H2" s="6" t="s">
-        <v>213</v>
+        <v>274</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>214</v>
+        <v>275</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>215</v>
+        <v>276</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>216</v>
+        <v>277</v>
       </c>
       <c r="L2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>217</v>
+        <v>278</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>46289</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>218</v>
+        <v>279</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>219</v>
+        <v>280</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>114</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>220</v>
+        <v>281</v>
       </c>
       <c r="G3" s="9"/>
       <c r="H3" s="9" t="s">
-        <v>221</v>
+        <v>282</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>222</v>
+        <v>283</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>223</v>
+        <v>284</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>224</v>
+        <v>285</v>
       </c>
       <c r="L3" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>225</v>
+        <v>286</v>
       </c>
       <c r="B4" s="10" t="n">
         <v>46289</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>226</v>
+        <v>287</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>227</v>
+        <v>288</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>131</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>228</v>
+        <v>289</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>229</v>
+        <v>290</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>230</v>
+        <v>291</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>231</v>
+        <v>292</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>232</v>
+        <v>293</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>216</v>
+        <v>277</v>
       </c>
       <c r="L4" s="9"/>
     </row>
@@ -4157,26 +5534,26 @@
         <v>46290</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>210</v>
+        <v>271</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>233</v>
+        <v>294</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>166</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>234</v>
+        <v>295</v>
       </c>
       <c r="G5" s="9"/>
       <c r="H5" s="9" t="s">
-        <v>235</v>
+        <v>296</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>236</v>
+        <v>297</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>237</v>
+        <v>298</v>
       </c>
       <c r="K5" s="9" t="s">
         <v>52</v>
@@ -4185,32 +5562,32 @@
     </row>
     <row r="6" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>238</v>
+        <v>299</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>46290</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>210</v>
+        <v>271</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>233</v>
+        <v>294</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>166</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>234</v>
+        <v>295</v>
       </c>
       <c r="G6" s="9"/>
       <c r="H6" s="9" t="s">
-        <v>235</v>
+        <v>296</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>236</v>
+        <v>297</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>239</v>
+        <v>300</v>
       </c>
       <c r="K6" s="9" t="s">
         <v>52</v>
@@ -4245,7 +5622,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="56"/>
@@ -4261,39 +5638,39 @@
         <v>28</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>240</v>
+        <v>301</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>241</v>
+        <v>302</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>242</v>
+        <v>303</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>243</v>
+        <v>304</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>244</v>
+        <v>305</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>245</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>212</v>
+        <v>273</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>246</v>
+        <v>307</v>
       </c>
       <c r="C2" s="6" t="n">
         <v>460676</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>247</v>
+        <v>308</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>248</v>
+        <v>309</v>
       </c>
       <c r="F2" s="7" t="n">
         <v>46287</v>
@@ -4305,16 +5682,16 @@
         <v>72</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>249</v>
+        <v>310</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>365</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>250</v>
+        <v>311</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>251</v>
+        <v>312</v>
       </c>
       <c r="F3" s="7" t="n">
         <v>46287</v>
@@ -4326,16 +5703,16 @@
         <v>76</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>252</v>
+        <v>313</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>415</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>253</v>
+        <v>314</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>254</v>
+        <v>315</v>
       </c>
       <c r="F4" s="7" t="n">
         <v>46287</v>
@@ -4347,16 +5724,16 @@
         <v>80</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>255</v>
+        <v>316</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>420</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>256</v>
+        <v>317</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>257</v>
+        <v>318</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>46287</v>
@@ -4365,19 +5742,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>258</v>
+        <v>319</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>246</v>
+        <v>307</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>192</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>259</v>
+        <v>320</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>260</v>
+        <v>321</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>46288</v>
@@ -4386,19 +5763,19 @@
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>261</v>
+        <v>322</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>262</v>
+        <v>323</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>22802</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>263</v>
+        <v>324</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>264</v>
+        <v>325</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>46288</v>
@@ -4407,19 +5784,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>265</v>
+        <v>326</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>266</v>
+        <v>327</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>9524</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>267</v>
+        <v>328</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>268</v>
+        <v>329</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>46288</v>
@@ -4431,16 +5808,16 @@
         <v>98</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>269</v>
+        <v>330</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>13590</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>270</v>
+        <v>331</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>271</v>
+        <v>332</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>46288</v>
@@ -4449,19 +5826,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>228</v>
+        <v>289</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>246</v>
+        <v>307</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>468785</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>272</v>
+        <v>333</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>273</v>
+        <v>334</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>46289</v>
@@ -4470,19 +5847,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>220</v>
+        <v>281</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>262</v>
+        <v>323</v>
       </c>
       <c r="C11" s="9" t="n">
         <v>48765</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>274</v>
+        <v>335</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>275</v>
+        <v>336</v>
       </c>
       <c r="F11" s="10" t="n">
         <v>46289</v>
@@ -4494,16 +5871,16 @@
         <v>119</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>269</v>
+        <v>330</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>9337</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>276</v>
+        <v>337</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>277</v>
+        <v>338</v>
       </c>
       <c r="F12" s="10" t="n">
         <v>46289</v>
@@ -4515,16 +5892,16 @@
         <v>124</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>266</v>
+        <v>327</v>
       </c>
       <c r="C13" s="9" t="n">
         <v>2868</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>278</v>
+        <v>339</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>279</v>
+        <v>340</v>
       </c>
       <c r="F13" s="10" t="n">
         <v>46289</v>
@@ -4533,19 +5910,19 @@
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>280</v>
+        <v>341</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>141791</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>282</v>
+        <v>343</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>283</v>
+        <v>344</v>
       </c>
       <c r="F14" s="10" t="n">
         <v>46289</v>
@@ -4557,16 +5934,16 @@
         <v>140</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>266</v>
+        <v>327</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>1416</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>284</v>
+        <v>345</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>285</v>
+        <v>346</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>46289</v>
@@ -4578,16 +5955,16 @@
         <v>144</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>269</v>
+        <v>330</v>
       </c>
       <c r="C16" s="9" t="n">
         <v>2595</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>286</v>
+        <v>347</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>287</v>
+        <v>348</v>
       </c>
       <c r="F16" s="10" t="n">
         <v>46289</v>
@@ -4596,19 +5973,19 @@
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>288</v>
+        <v>349</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>266</v>
+        <v>327</v>
       </c>
       <c r="C17" s="9" t="n">
         <v>18407</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>289</v>
+        <v>350</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>290</v>
+        <v>351</v>
       </c>
       <c r="F17" s="10" t="n">
         <v>46290</v>
@@ -4617,19 +5994,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>291</v>
+        <v>352</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>262</v>
+        <v>323</v>
       </c>
       <c r="C18" s="9" t="n">
         <v>51730</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>292</v>
+        <v>353</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>293</v>
+        <v>354</v>
       </c>
       <c r="F18" s="10" t="n">
         <v>46290</v>
@@ -4638,19 +6015,19 @@
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>294</v>
+        <v>355</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C19" s="9" t="n">
         <v>150866</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>295</v>
+        <v>356</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>296</v>
+        <v>357</v>
       </c>
       <c r="F19" s="10" t="n">
         <v>46290</v>
@@ -4659,19 +6036,19 @@
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>297</v>
+        <v>358</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>227085</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>298</v>
+        <v>359</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>299</v>
+        <v>360</v>
       </c>
       <c r="F20" s="10" t="n">
         <v>46290</v>
@@ -4680,19 +6057,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>300</v>
+        <v>361</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C21" s="9" t="n">
         <v>70321</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>301</v>
+        <v>362</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>302</v>
+        <v>363</v>
       </c>
       <c r="F21" s="10" t="n">
         <v>46290</v>
@@ -4701,19 +6078,19 @@
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>303</v>
+        <v>364</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C22" s="9" t="n">
         <v>440073</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>304</v>
+        <v>365</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>305</v>
+        <v>366</v>
       </c>
       <c r="F22" s="10" t="n">
         <v>46290</v>
@@ -4722,19 +6099,19 @@
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>306</v>
+        <v>367</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>263530</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>307</v>
+        <v>368</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>308</v>
+        <v>369</v>
       </c>
       <c r="F23" s="10" t="n">
         <v>46290</v>
@@ -4743,19 +6120,19 @@
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>309</v>
+        <v>370</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C24" s="9" t="n">
         <v>63054</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>310</v>
+        <v>371</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>311</v>
+        <v>372</v>
       </c>
       <c r="F24" s="10" t="n">
         <v>46290</v>
@@ -4764,19 +6141,19 @@
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>312</v>
+        <v>373</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C25" s="9" t="n">
         <v>373125</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>313</v>
+        <v>374</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>314</v>
+        <v>375</v>
       </c>
       <c r="F25" s="10" t="n">
         <v>46290</v>
@@ -4785,19 +6162,19 @@
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>315</v>
+        <v>376</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C26" s="9" t="n">
         <v>202395</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>316</v>
+        <v>377</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>317</v>
+        <v>378</v>
       </c>
       <c r="F26" s="10" t="n">
         <v>46290</v>
@@ -4806,19 +6183,19 @@
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>318</v>
+        <v>379</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C27" s="9" t="n">
         <v>17992</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>319</v>
+        <v>380</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>320</v>
+        <v>381</v>
       </c>
       <c r="F27" s="10" t="n">
         <v>46290</v>
@@ -4827,19 +6204,19 @@
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>321</v>
+        <v>382</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="C28" s="9" t="n">
         <v>108430</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>322</v>
+        <v>383</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>323</v>
+        <v>384</v>
       </c>
       <c r="F28" s="10" t="n">
         <v>46290</v>
@@ -4851,16 +6228,16 @@
         <v>177</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>269</v>
+        <v>330</v>
       </c>
       <c r="C29" s="9" t="n">
         <v>2667</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>324</v>
+        <v>385</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>325</v>
+        <v>386</v>
       </c>
       <c r="F29" s="10" t="n">
         <v>46290</v>
@@ -4869,19 +6246,19 @@
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>234</v>
+        <v>295</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>266</v>
+        <v>327</v>
       </c>
       <c r="C30" s="9" t="n">
         <v>19801</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>326</v>
+        <v>387</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>327</v>
+        <v>388</v>
       </c>
       <c r="F30" s="10" t="n">
         <v>46290</v>
@@ -4890,19 +6267,19 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>328</v>
+        <v>389</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>262</v>
+        <v>323</v>
       </c>
       <c r="C31" s="9" t="n">
         <v>70580</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>329</v>
+        <v>390</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>330</v>
+        <v>391</v>
       </c>
       <c r="F31" s="10" t="n">
         <v>46290</v>
@@ -4914,42 +6291,462 @@
         <v>194</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>269</v>
+        <v>330</v>
       </c>
       <c r="C32" s="9" t="n">
         <v>13093</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>331</v>
+        <v>392</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>332</v>
+        <v>393</v>
       </c>
       <c r="F32" s="10" t="n">
         <v>46290</v>
       </c>
       <c r="G32" s="9"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
         <v>198</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>269</v>
+        <v>330</v>
       </c>
       <c r="C33" s="9" t="n">
         <v>2580</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>333</v>
+        <v>394</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>334</v>
+        <v>395</v>
       </c>
       <c r="F33" s="10" t="n">
         <v>46290</v>
       </c>
       <c r="G33" s="9"/>
+    </row>
+    <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>400646</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="F34" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G34" s="9"/>
+    </row>
+    <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>13150</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="F35" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G35" s="9"/>
+    </row>
+    <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="s">
+        <v>403</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>323</v>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>11135</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="F36" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G36" s="9"/>
+    </row>
+    <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>1640514</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="F37" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="9" t="s">
+        <v>409</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="C38" s="9" t="n">
+        <v>354138</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="F38" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G38" s="9"/>
+    </row>
+    <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="C39" s="9" t="n">
+        <v>354683</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>413</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C40" s="9" t="n">
+        <v>23697</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>416</v>
+      </c>
+      <c r="F40" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G40" s="9"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C41" s="9" t="n">
+        <v>7023</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>418</v>
+      </c>
+      <c r="F41" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C42" s="9" t="n">
+        <v>21297</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>419</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="F42" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G42" s="9"/>
+    </row>
+    <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>21297</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>419</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="F43" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C44" s="9" t="n">
+        <v>7023</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="F44" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G44" s="9"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C45" s="9" t="n">
+        <v>13590</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>331</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="F45" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C46" s="9" t="n">
+        <v>9337</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>337</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="F46" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G46" s="9"/>
+    </row>
+    <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C47" s="9" t="n">
+        <v>2595</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>347</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="F47" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C48" s="9" t="n">
+        <v>2580</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>394</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>426</v>
+      </c>
+      <c r="F48" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G48" s="9"/>
+    </row>
+    <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C49" s="9" t="n">
+        <v>13093</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>392</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="F49" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C50" s="9" t="n">
+        <v>2667</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="F50" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G50" s="9"/>
+    </row>
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C51" s="9" t="n">
+        <v>3400</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>429</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="F51" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="C52" s="9" t="n">
+        <v>23697</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="F52" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G52" s="9"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>327</v>
+      </c>
+      <c r="C53" s="9" t="n">
+        <v>4533</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>432</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="F53" s="10" t="n">
+        <v>46291</v>
+      </c>
+      <c r="G53" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
@@ -5003,88 +6800,88 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>335</v>
+        <v>434</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>202</v>
+        <v>263</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>336</v>
+        <v>435</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>337</v>
+        <v>436</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>338</v>
+        <v>437</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>339</v>
+        <v>438</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>340</v>
+        <v>439</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>341</v>
+        <v>440</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>342</v>
+        <v>441</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>343</v>
+        <v>442</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>344</v>
+        <v>443</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>345</v>
+        <v>444</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>346</v>
+        <v>445</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>347</v>
+        <v>446</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>348</v>
+        <v>447</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>349</v>
+        <v>448</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>350</v>
+        <v>449</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>351</v>
+        <v>450</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>352</v>
+        <v>451</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>353</v>
+        <v>452</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>354</v>
+        <v>453</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>355</v>
+        <v>454</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>356</v>
+        <v>455</v>
       </c>
       <c r="Y1" s="5" t="s">
-        <v>357</v>
+        <v>456</v>
       </c>
       <c r="Z1" s="5" t="s">
-        <v>358</v>
+        <v>457</v>
       </c>
       <c r="AA1" s="5" t="s">
         <v>11</v>
       </c>
       <c r="AB1" s="5" t="s">
-        <v>208</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -5121,7 +6918,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>359</v>
+        <v>458</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -5137,15 +6934,15 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>360</v>
+        <v>459</v>
       </c>
       <c r="B3" s="13" t="n">
         <f aca="false">COUNTA(Change_Log!A2:A5000)</f>
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13" t="s">
-        <v>361</v>
+        <v>460</v>
       </c>
       <c r="E3" s="13" t="n">
         <f aca="false">COUNTA(Experiments!A2:A5000)</f>
@@ -5154,7 +6951,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>362</v>
+        <v>461</v>
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">COUNTA(Findings!A2:A5000)</f>
@@ -5162,7 +6959,7 @@
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13" t="s">
-        <v>363</v>
+        <v>462</v>
       </c>
       <c r="E4" s="13" t="n">
         <f aca="false">COUNTIF(Experiments!AA2:AA5000,"Done")</f>
@@ -5171,7 +6968,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>364</v>
+        <v>463</v>
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">COUNTIF(Findings!K2:K5000,"Open")</f>
@@ -5179,7 +6976,7 @@
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13" t="s">
-        <v>365</v>
+        <v>464</v>
       </c>
       <c r="E5" s="13" t="n">
         <f aca="false">COUNTIF(Experiments!AA2:AA5000,"Failed")</f>
@@ -5195,7 +6992,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>366</v>
+        <v>465</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -5204,7 +7001,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>367</v>
+        <v>466</v>
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A8)</f>
@@ -5216,7 +7013,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>368</v>
+        <v>467</v>
       </c>
       <c r="B9" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A9)</f>
@@ -5232,7 +7029,7 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A10)</f>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
@@ -5244,7 +7041,7 @@
       </c>
       <c r="B11" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A11)</f>
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
@@ -5256,7 +7053,7 @@
       </c>
       <c r="B12" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A12)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
@@ -5264,7 +7061,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>369</v>
+        <v>468</v>
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A13)</f>
@@ -5280,7 +7077,7 @@
       </c>
       <c r="B14" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A14)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
@@ -5292,7 +7089,7 @@
       </c>
       <c r="B15" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!I2:I5000,A15)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
@@ -5331,7 +7128,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>370</v>
+        <v>469</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -5344,7 +7141,7 @@
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!S2:S5000,A20)</f>
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
@@ -5352,7 +7149,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>216</v>
+        <v>277</v>
       </c>
       <c r="B21" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!S2:S5000,A21)</f>
@@ -5364,7 +7161,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>371</v>
+        <v>470</v>
       </c>
       <c r="B22" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!S2:S5000,A22)</f>
@@ -5376,7 +7173,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>372</v>
+        <v>471</v>
       </c>
       <c r="B23" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!S2:S5000,A23)</f>
@@ -5388,7 +7185,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>224</v>
+        <v>285</v>
       </c>
       <c r="B24" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!S2:S5000,A24)</f>
@@ -5407,7 +7204,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>373</v>
+        <v>472</v>
       </c>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
@@ -5420,7 +7217,7 @@
       </c>
       <c r="B27" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!R2:R5000,A27)</f>
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
@@ -5428,7 +7225,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>218</v>
+        <v>279</v>
       </c>
       <c r="B28" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!R2:R5000,A28)</f>
@@ -5440,7 +7237,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>210</v>
+        <v>271</v>
       </c>
       <c r="B29" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!R2:R5000,A29)</f>
@@ -5452,7 +7249,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>226</v>
+        <v>287</v>
       </c>
       <c r="B30" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!R2:R5000,A30)</f>
@@ -5464,7 +7261,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>374</v>
+        <v>473</v>
       </c>
       <c r="B31" s="13" t="n">
         <f aca="false">COUNTIF(Change_Log!R2:R5000,A31)</f>

</xml_diff>